<commit_message>
Update costing output for 2026-03-26
</commit_message>
<xml_diff>
--- a/output/2026-03-26/20260326_Costing TMT.xlsx
+++ b/output/2026-03-26/20260326_Costing TMT.xlsx
@@ -1,20 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17500" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Raipur" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="NCR" sheetId="2" state="visible" r:id="rId2"/>
-  </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
-</workbook>
+<s:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <s:workbookPr/>
+  <s:bookViews>
+    <s:workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17500" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+  </s:bookViews>
+  <s:sheets>
+    <s:sheet name="Raipur" sheetId="1" state="visible" r:id="rId1"/>
+    <s:sheet name="NCR" sheetId="2" state="visible" r:id="rId2"/>
+  </s:sheets>
+  <s:definedNames/>
+  <s:calcPr calcId="191029" fullCalcOnLoad="1"/>
+</s:workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1428,82 +1425,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Sumit K</author>
-  </authors>
-  <commentList>
-    <comment ref="B10" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Sumit K:
-25-150 mm, HC 60-14 
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Sumit K</author>
-  </authors>
-  <commentList>
-    <comment ref="A10" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Sumit K:
-25-150 mm, HC 60-14 
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
-    <sheetNames>
-      <sheetName val="Sheet1"/>
-      <sheetName val="Sheet2"/>
-      <sheetName val="Steel Mint Inputs"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="53">
-          <cell r="F53">
-            <v>41582.325872340429</v>
-          </cell>
-          <cell r="O53">
-            <v>44443.723852410454</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="F54">
-            <v>42000</v>
-          </cell>
-          <cell r="O54">
-            <v>45500</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="F55">
-            <v>417.67412765957124</v>
-          </cell>
-          <cell r="O55">
-            <v>1056.2761475895459</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3094,7 +3015,6 @@
   <colBreaks count="1" manualBreakCount="1">
     <brk id="25" min="0" max="54" man="1"/>
   </colBreaks>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -3944,6 +3864,5 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>